<commit_message>
Bo sung tinh nang phieu xuat dieu chuyen
</commit_message>
<xml_diff>
--- a/Data/MaKho.xlsx
+++ b/Data/MaKho.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dropbox\Works 2\IT\GITHUB\UpSSE_BB\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{133AEF97-6B80-4D42-B37C-F9C109F06D31}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F27D4205-EEFF-4D98-95F4-CABB8A3C8EBC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,144 +39,36 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="88">
   <si>
-    <t>Bến xe phía Bắc</t>
-  </si>
-  <si>
-    <t>Đại An</t>
-  </si>
-  <si>
-    <t>Cộng Hoà</t>
-  </si>
-  <si>
     <t>KDNL005</t>
   </si>
   <si>
     <t>KDNL006</t>
   </si>
   <si>
-    <t>Đông Ninh Phúc</t>
-  </si>
-  <si>
-    <t>Đông Thi Sơn</t>
-  </si>
-  <si>
-    <t>Gia Thanh</t>
-  </si>
-  <si>
-    <t>Gia Xuân</t>
-  </si>
-  <si>
-    <t>Giao Thủy</t>
-  </si>
-  <si>
-    <t>Hải Vân</t>
-  </si>
-  <si>
     <t>KDNL053</t>
   </si>
   <si>
-    <t>Hồng Sơn</t>
-  </si>
-  <si>
-    <t>Hùng Vương</t>
-  </si>
-  <si>
     <t>KDNL063</t>
   </si>
   <si>
-    <t>Khánh Hòa</t>
-  </si>
-  <si>
-    <t>Khánh Ninh</t>
-  </si>
-  <si>
-    <t>Liêm Phong</t>
-  </si>
-  <si>
-    <t>Liên Minh</t>
-  </si>
-  <si>
-    <t>Liễu Đề</t>
-  </si>
-  <si>
-    <t>Lộc An</t>
-  </si>
-  <si>
     <t>KDNL051</t>
   </si>
   <si>
-    <t>Lộc Hạ</t>
-  </si>
-  <si>
     <t>KDNL004</t>
   </si>
   <si>
-    <t>Mỹ Lộc</t>
-  </si>
-  <si>
-    <t>Mỹ Xá</t>
-  </si>
-  <si>
     <t>KDNL003</t>
   </si>
   <si>
-    <t>Nam Hồng</t>
-  </si>
-  <si>
     <t>KDNL018</t>
   </si>
   <si>
-    <t>Nam Vân</t>
-  </si>
-  <si>
-    <t>Nguyễn Huệ</t>
-  </si>
-  <si>
-    <t>Nhân Chính</t>
-  </si>
-  <si>
-    <t>Ninh Giang</t>
-  </si>
-  <si>
-    <t>Phủ Lý</t>
-  </si>
-  <si>
-    <t>Quảng Trường</t>
-  </si>
-  <si>
-    <t>Song Hào</t>
-  </si>
-  <si>
     <t>KDNL065</t>
   </si>
   <si>
-    <t>Tam Điệp</t>
-  </si>
-  <si>
-    <t>Tân Thành</t>
-  </si>
-  <si>
-    <t>Thanh Phong</t>
-  </si>
-  <si>
-    <t>Trạm cấp</t>
-  </si>
-  <si>
     <t>KHO4</t>
   </si>
   <si>
-    <t>Tràng An</t>
-  </si>
-  <si>
-    <t>Trì Chính</t>
-  </si>
-  <si>
-    <t>Văn Phong</t>
-  </si>
-  <si>
-    <t>Xuân Trường</t>
-  </si>
-  <si>
     <t>KDNL011</t>
   </si>
   <si>
@@ -255,52 +147,160 @@
     <t>KDNL175</t>
   </si>
   <si>
-    <t>Đại Hoàng</t>
-  </si>
-  <si>
     <t>KDNL178</t>
   </si>
   <si>
-    <t>Hoa Lư</t>
-  </si>
-  <si>
     <t>KDNL179</t>
   </si>
   <si>
-    <t>Bái Đính</t>
-  </si>
-  <si>
     <t>KDNL177</t>
   </si>
   <si>
-    <t>Gia Tường</t>
-  </si>
-  <si>
     <t>KDNL080</t>
   </si>
   <si>
-    <t>Tiên Tân</t>
-  </si>
-  <si>
     <t>KDNL183</t>
   </si>
   <si>
-    <t>Châu Sơn</t>
-  </si>
-  <si>
     <t>KDNL182</t>
   </si>
   <si>
-    <t>Quất Lâm</t>
-  </si>
-  <si>
     <t>KDNL081</t>
   </si>
   <si>
-    <t>Thiên Tôn</t>
-  </si>
-  <si>
     <t>KDNL184</t>
+  </si>
+  <si>
+    <t>CHXD Bến xe phía Bắc</t>
+  </si>
+  <si>
+    <t>CHXD Cộng Hoà</t>
+  </si>
+  <si>
+    <t>CHXD Đại An</t>
+  </si>
+  <si>
+    <t>CHXD Đông Ninh Phúc</t>
+  </si>
+  <si>
+    <t>CHXD Đông Thi Sơn</t>
+  </si>
+  <si>
+    <t>CHXD Gia Thanh</t>
+  </si>
+  <si>
+    <t>CHXD Gia Xuân</t>
+  </si>
+  <si>
+    <t>CHXD Giao Thủy</t>
+  </si>
+  <si>
+    <t>CHXD Hải Vân</t>
+  </si>
+  <si>
+    <t>CHXD Hồng Sơn</t>
+  </si>
+  <si>
+    <t>CHXD Hùng Vương</t>
+  </si>
+  <si>
+    <t>CHXD Khánh Hòa</t>
+  </si>
+  <si>
+    <t>CHXD Khánh Ninh</t>
+  </si>
+  <si>
+    <t>CHXD Liêm Phong</t>
+  </si>
+  <si>
+    <t>CHXD Liên Minh</t>
+  </si>
+  <si>
+    <t>CHXD Liễu Đề</t>
+  </si>
+  <si>
+    <t>CHXD Lộc An</t>
+  </si>
+  <si>
+    <t>CHXD Lộc Hạ</t>
+  </si>
+  <si>
+    <t>CHXD Mỹ Lộc</t>
+  </si>
+  <si>
+    <t>CHXD Mỹ Xá</t>
+  </si>
+  <si>
+    <t>CHXD Nam Hồng</t>
+  </si>
+  <si>
+    <t>CHXD Nam Vân</t>
+  </si>
+  <si>
+    <t>CHXD Nguyễn Huệ</t>
+  </si>
+  <si>
+    <t>CHXD Nhân Chính</t>
+  </si>
+  <si>
+    <t>CHXD Ninh Giang</t>
+  </si>
+  <si>
+    <t>CHXD Phủ Lý</t>
+  </si>
+  <si>
+    <t>CHXD Quảng Trường</t>
+  </si>
+  <si>
+    <t>CHXD Song Hào</t>
+  </si>
+  <si>
+    <t>CHXD Tam Điệp</t>
+  </si>
+  <si>
+    <t>CHXD Tân Thành</t>
+  </si>
+  <si>
+    <t>CHXD Thanh Phong</t>
+  </si>
+  <si>
+    <t>CHXD Trạm cấp</t>
+  </si>
+  <si>
+    <t>CHXD Tràng An</t>
+  </si>
+  <si>
+    <t>CHXD Trì Chính</t>
+  </si>
+  <si>
+    <t>CHXD Văn Phong</t>
+  </si>
+  <si>
+    <t>CHXD Xuân Trường</t>
+  </si>
+  <si>
+    <t>CHXD Đại Hoàng</t>
+  </si>
+  <si>
+    <t>CHXD Hoa Lư</t>
+  </si>
+  <si>
+    <t>CHXD Bái Đính</t>
+  </si>
+  <si>
+    <t>CHXD Gia Tường</t>
+  </si>
+  <si>
+    <t>CHXD Tiên Tân</t>
+  </si>
+  <si>
+    <t>CHXD Châu Sơn</t>
+  </si>
+  <si>
+    <t>CHXD Quất Lâm</t>
+  </si>
+  <si>
+    <t>CHXD Thiên Tôn</t>
   </si>
 </sst>
 </file>
@@ -761,367 +761,367 @@
   <sheetData>
     <row r="1" spans="1:4" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>0</v>
+        <v>44</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>52</v>
+        <v>16</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>2</v>
+        <v>45</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="B3" s="1" t="s">
         <v>1</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>4</v>
       </c>
     </row>
     <row r="4" spans="1:4" s="5" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>5</v>
+        <v>47</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>53</v>
+        <v>17</v>
       </c>
       <c r="C4" s="1"/>
       <c r="D4" s="1"/>
     </row>
     <row r="5" spans="1:4" s="5" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>6</v>
+        <v>48</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>54</v>
+        <v>18</v>
       </c>
       <c r="C5" s="1"/>
       <c r="D5" s="1"/>
     </row>
     <row r="6" spans="1:4" s="5" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
-        <v>7</v>
+        <v>49</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>55</v>
+        <v>19</v>
       </c>
       <c r="C6" s="1"/>
       <c r="D6" s="1"/>
     </row>
     <row r="7" spans="1:4" s="5" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
-        <v>8</v>
+        <v>50</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>56</v>
+        <v>20</v>
       </c>
       <c r="C7" s="1"/>
       <c r="D7" s="1"/>
     </row>
     <row r="8" spans="1:4" s="5" customFormat="1" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
-        <v>9</v>
+        <v>51</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>46</v>
+        <v>10</v>
       </c>
       <c r="D8" s="1"/>
     </row>
     <row r="9" spans="1:4" s="5" customFormat="1" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
-        <v>10</v>
+        <v>52</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="D9" s="1"/>
     </row>
     <row r="10" spans="1:4" s="5" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
-        <v>12</v>
+        <v>53</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>57</v>
+        <v>21</v>
       </c>
       <c r="D10" s="1"/>
     </row>
     <row r="11" spans="1:4" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
-        <v>13</v>
+        <v>54</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>14</v>
+        <v>3</v>
       </c>
       <c r="C11" s="5"/>
     </row>
     <row r="12" spans="1:4" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
-        <v>15</v>
+        <v>55</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>58</v>
+        <v>22</v>
       </c>
     </row>
     <row r="13" spans="1:4" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
-        <v>16</v>
+        <v>56</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>59</v>
+        <v>23</v>
       </c>
     </row>
     <row r="14" spans="1:4" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
-        <v>17</v>
+        <v>57</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>60</v>
+        <v>24</v>
       </c>
     </row>
     <row r="15" spans="1:4" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
-        <v>18</v>
+        <v>58</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>47</v>
+        <v>11</v>
       </c>
     </row>
     <row r="16" spans="1:4" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
-        <v>19</v>
+        <v>59</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>48</v>
+        <v>12</v>
       </c>
     </row>
     <row r="17" spans="1:3" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
-        <v>20</v>
+        <v>60</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>21</v>
+        <v>4</v>
       </c>
     </row>
     <row r="18" spans="1:3" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
-        <v>22</v>
+        <v>61</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>23</v>
+        <v>5</v>
       </c>
     </row>
     <row r="19" spans="1:3" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
-        <v>24</v>
+        <v>62</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>49</v>
+        <v>13</v>
       </c>
     </row>
     <row r="20" spans="1:3" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
-        <v>25</v>
+        <v>63</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>26</v>
+        <v>6</v>
       </c>
     </row>
     <row r="21" spans="1:3" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="3" t="s">
-        <v>27</v>
+        <v>64</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>28</v>
+        <v>7</v>
       </c>
     </row>
     <row r="22" spans="1:3" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="3" t="s">
-        <v>29</v>
+        <v>65</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>50</v>
+        <v>14</v>
       </c>
     </row>
     <row r="23" spans="1:3" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="3" t="s">
-        <v>30</v>
+        <v>66</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>61</v>
+        <v>25</v>
       </c>
       <c r="C23" s="2"/>
     </row>
     <row r="24" spans="1:3" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="3" t="s">
-        <v>31</v>
+        <v>67</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>62</v>
+        <v>26</v>
       </c>
     </row>
     <row r="25" spans="1:3" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="3" t="s">
-        <v>32</v>
+        <v>68</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>63</v>
+        <v>27</v>
       </c>
     </row>
     <row r="26" spans="1:3" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="3" t="s">
-        <v>33</v>
+        <v>69</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>64</v>
+        <v>28</v>
       </c>
     </row>
     <row r="27" spans="1:3" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="3" t="s">
-        <v>34</v>
+        <v>70</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>65</v>
+        <v>29</v>
       </c>
     </row>
     <row r="28" spans="1:3" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="3" t="s">
-        <v>35</v>
+        <v>71</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>36</v>
+        <v>8</v>
       </c>
     </row>
     <row r="29" spans="1:3" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="3" t="s">
-        <v>37</v>
+        <v>72</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>66</v>
+        <v>30</v>
       </c>
     </row>
     <row r="30" spans="1:3" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="3" t="s">
-        <v>38</v>
+        <v>73</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>67</v>
+        <v>31</v>
       </c>
     </row>
     <row r="31" spans="1:3" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="3" t="s">
-        <v>39</v>
+        <v>74</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>68</v>
+        <v>32</v>
       </c>
     </row>
     <row r="32" spans="1:3" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="3" t="s">
-        <v>40</v>
+        <v>75</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>41</v>
+        <v>9</v>
       </c>
     </row>
     <row r="33" spans="1:2" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="3" t="s">
-        <v>42</v>
+        <v>76</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>69</v>
+        <v>33</v>
       </c>
     </row>
     <row r="34" spans="1:2" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="3" t="s">
-        <v>43</v>
+        <v>77</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>70</v>
+        <v>34</v>
       </c>
     </row>
     <row r="35" spans="1:2" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="3" t="s">
-        <v>44</v>
+        <v>78</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>71</v>
+        <v>35</v>
       </c>
     </row>
     <row r="36" spans="1:2" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="3" t="s">
-        <v>45</v>
+        <v>79</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>51</v>
+        <v>15</v>
       </c>
     </row>
     <row r="37" spans="1:2" ht="9.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="3" t="s">
-        <v>72</v>
+        <v>80</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>73</v>
+        <v>36</v>
       </c>
     </row>
     <row r="38" spans="1:2" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="1" t="s">
-        <v>74</v>
+        <v>81</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>75</v>
+        <v>37</v>
       </c>
     </row>
     <row r="39" spans="1:2" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="1" t="s">
-        <v>76</v>
+        <v>82</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>77</v>
+        <v>38</v>
       </c>
     </row>
     <row r="40" spans="1:2" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="1" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>79</v>
+        <v>39</v>
       </c>
     </row>
     <row r="41" spans="1:2" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="1" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>81</v>
+        <v>40</v>
       </c>
     </row>
     <row r="42" spans="1:2" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="1" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>83</v>
+        <v>41</v>
       </c>
     </row>
     <row r="43" spans="1:2" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="1" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>85</v>
+        <v>42</v>
       </c>
     </row>
     <row r="44" spans="1:2" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="1" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>87</v>
+        <v>43</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Điều chỉnh tên kho Nam Định
</commit_message>
<xml_diff>
--- a/Data/MaKho.xlsx
+++ b/Data/MaKho.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dropbox\Works 2\IT\GITHUB\UpSSE_BB\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F27D4205-EEFF-4D98-95F4-CABB8A3C8EBC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FCAE31D6-FBB0-46D3-BBFE-C0A2EC44B145}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="92">
   <si>
     <t>KDNL005</t>
   </si>
@@ -165,9 +165,6 @@
     <t>KDNL182</t>
   </si>
   <si>
-    <t>KDNL081</t>
-  </si>
-  <si>
     <t>KDNL184</t>
   </si>
   <si>
@@ -301,6 +298,21 @@
   </si>
   <si>
     <t>CHXD Thiên Tôn</t>
+  </si>
+  <si>
+    <t>KDNL181</t>
+  </si>
+  <si>
+    <t>CHXD Hợp Hưng</t>
+  </si>
+  <si>
+    <t>KDNL185</t>
+  </si>
+  <si>
+    <t>CHXD Trường Thi</t>
+  </si>
+  <si>
+    <t>KDNL186</t>
   </si>
 </sst>
 </file>
@@ -751,17 +763,17 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:D44"/>
+  <dimension ref="A1:D46"/>
   <sheetFormatPr defaultColWidth="8.42578125" defaultRowHeight="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="15.7109375" style="1" customWidth="1"/>
+    <col min="1" max="1" width="21.7109375" style="1" customWidth="1"/>
     <col min="2" max="378" width="8.42578125" style="1" customWidth="1"/>
     <col min="379" max="16384" width="8.42578125" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>16</v>
@@ -769,7 +781,7 @@
     </row>
     <row r="2" spans="1:4" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>0</v>
@@ -777,7 +789,7 @@
     </row>
     <row r="3" spans="1:4" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>1</v>
@@ -785,7 +797,7 @@
     </row>
     <row r="4" spans="1:4" s="5" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>17</v>
@@ -795,7 +807,7 @@
     </row>
     <row r="5" spans="1:4" s="5" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B5" s="1" t="s">
         <v>18</v>
@@ -805,7 +817,7 @@
     </row>
     <row r="6" spans="1:4" s="5" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>19</v>
@@ -815,7 +827,7 @@
     </row>
     <row r="7" spans="1:4" s="5" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>20</v>
@@ -825,7 +837,7 @@
     </row>
     <row r="8" spans="1:4" s="5" customFormat="1" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B8" s="5" t="s">
         <v>10</v>
@@ -834,7 +846,7 @@
     </row>
     <row r="9" spans="1:4" s="5" customFormat="1" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B9" s="5" t="s">
         <v>2</v>
@@ -843,7 +855,7 @@
     </row>
     <row r="10" spans="1:4" s="5" customFormat="1" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B10" s="5" t="s">
         <v>21</v>
@@ -852,7 +864,7 @@
     </row>
     <row r="11" spans="1:4" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B11" s="5" t="s">
         <v>3</v>
@@ -861,7 +873,7 @@
     </row>
     <row r="12" spans="1:4" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B12" s="1" t="s">
         <v>22</v>
@@ -869,7 +881,7 @@
     </row>
     <row r="13" spans="1:4" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B13" s="1" t="s">
         <v>23</v>
@@ -877,7 +889,7 @@
     </row>
     <row r="14" spans="1:4" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B14" s="1" t="s">
         <v>24</v>
@@ -885,7 +897,7 @@
     </row>
     <row r="15" spans="1:4" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B15" s="1" t="s">
         <v>11</v>
@@ -893,7 +905,7 @@
     </row>
     <row r="16" spans="1:4" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B16" s="1" t="s">
         <v>12</v>
@@ -901,7 +913,7 @@
     </row>
     <row r="17" spans="1:3" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B17" s="1" t="s">
         <v>4</v>
@@ -909,7 +921,7 @@
     </row>
     <row r="18" spans="1:3" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B18" s="1" t="s">
         <v>5</v>
@@ -917,7 +929,7 @@
     </row>
     <row r="19" spans="1:3" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B19" s="1" t="s">
         <v>13</v>
@@ -925,7 +937,7 @@
     </row>
     <row r="20" spans="1:3" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B20" s="1" t="s">
         <v>6</v>
@@ -933,7 +945,7 @@
     </row>
     <row r="21" spans="1:3" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="3" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B21" s="1" t="s">
         <v>7</v>
@@ -941,7 +953,7 @@
     </row>
     <row r="22" spans="1:3" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="3" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B22" s="1" t="s">
         <v>14</v>
@@ -949,7 +961,7 @@
     </row>
     <row r="23" spans="1:3" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="3" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B23" s="1" t="s">
         <v>25</v>
@@ -958,7 +970,7 @@
     </row>
     <row r="24" spans="1:3" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B24" s="1" t="s">
         <v>26</v>
@@ -966,7 +978,7 @@
     </row>
     <row r="25" spans="1:3" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B25" s="1" t="s">
         <v>27</v>
@@ -974,7 +986,7 @@
     </row>
     <row r="26" spans="1:3" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B26" s="1" t="s">
         <v>28</v>
@@ -982,7 +994,7 @@
     </row>
     <row r="27" spans="1:3" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="3" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B27" s="1" t="s">
         <v>29</v>
@@ -990,7 +1002,7 @@
     </row>
     <row r="28" spans="1:3" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="3" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B28" s="1" t="s">
         <v>8</v>
@@ -998,7 +1010,7 @@
     </row>
     <row r="29" spans="1:3" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="3" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B29" s="1" t="s">
         <v>30</v>
@@ -1006,7 +1018,7 @@
     </row>
     <row r="30" spans="1:3" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="3" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B30" s="1" t="s">
         <v>31</v>
@@ -1014,7 +1026,7 @@
     </row>
     <row r="31" spans="1:3" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="3" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B31" s="1" t="s">
         <v>32</v>
@@ -1022,7 +1034,7 @@
     </row>
     <row r="32" spans="1:3" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="3" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B32" s="1" t="s">
         <v>9</v>
@@ -1030,7 +1042,7 @@
     </row>
     <row r="33" spans="1:2" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="3" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B33" s="1" t="s">
         <v>33</v>
@@ -1038,7 +1050,7 @@
     </row>
     <row r="34" spans="1:2" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="3" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B34" s="1" t="s">
         <v>34</v>
@@ -1046,7 +1058,7 @@
     </row>
     <row r="35" spans="1:2" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="3" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B35" s="1" t="s">
         <v>35</v>
@@ -1054,7 +1066,7 @@
     </row>
     <row r="36" spans="1:2" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="3" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B36" s="1" t="s">
         <v>15</v>
@@ -1062,7 +1074,7 @@
     </row>
     <row r="37" spans="1:2" ht="9.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="3" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B37" s="1" t="s">
         <v>36</v>
@@ -1070,7 +1082,7 @@
     </row>
     <row r="38" spans="1:2" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="1" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B38" s="1" t="s">
         <v>37</v>
@@ -1078,7 +1090,7 @@
     </row>
     <row r="39" spans="1:2" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B39" s="1" t="s">
         <v>38</v>
@@ -1086,7 +1098,7 @@
     </row>
     <row r="40" spans="1:2" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B40" s="1" t="s">
         <v>39</v>
@@ -1094,7 +1106,7 @@
     </row>
     <row r="41" spans="1:2" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B41" s="1" t="s">
         <v>40</v>
@@ -1102,7 +1114,7 @@
     </row>
     <row r="42" spans="1:2" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="1" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B42" s="1" t="s">
         <v>41</v>
@@ -1110,18 +1122,34 @@
     </row>
     <row r="43" spans="1:2" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="1" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>42</v>
+        <v>87</v>
       </c>
     </row>
     <row r="44" spans="1:2" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="1" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
+      </c>
+    </row>
+    <row r="45" spans="1:2" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A45" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="B45" s="1" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="46" spans="1:2" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A46" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="B46" s="1" t="s">
+        <v>91</v>
       </c>
     </row>
   </sheetData>

</xml_diff>